<commit_message>
Regenerate the todays-fixes E2E fixtures from the current build
The two workbooks e2eTodaysFixes.mjs imports are generated at the start of
every run, so they carry the sale dates of the day they were produced. This
is that regeneration against a fresh VITE_E2E build — no schema or column
changes, only the dates and the zip's own timestamps moved.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/todays-fixes/fixtures/FIXVERIFY_INVENTORY.xlsx
+++ b/e2e-screenshots/todays-fixes/fixtures/FIXVERIFY_INVENTORY.xlsx
@@ -436,7 +436,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-06</v>
+        <v>2026-06-07</v>
       </c>
       <c r="B2" t="str">
         <v>FIXVERIFY 12</v>
@@ -471,7 +471,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-06-06</v>
+        <v>2026-06-07</v>
       </c>
       <c r="B3" t="str">
         <v>FIXVERIFY 12</v>
@@ -506,7 +506,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-06-06</v>
+        <v>2026-06-07</v>
       </c>
       <c r="B4" t="str">
         <v>FIXVERIFY 12</v>
@@ -541,7 +541,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-06-06</v>
+        <v>2026-06-07</v>
       </c>
       <c r="B5" t="str">
         <v>FIXVERIFY 15</v>
@@ -576,7 +576,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-06-06</v>
+        <v>2026-06-07</v>
       </c>
       <c r="B6" t="str">
         <v>FIXVERIFY 15</v>
@@ -611,7 +611,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-06-06</v>
+        <v>2026-06-07</v>
       </c>
       <c r="B7" t="str">
         <v>FIXVERIFY 15</v>
@@ -646,7 +646,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-06-06</v>
+        <v>2026-06-07</v>
       </c>
       <c r="B8" t="str">
         <v>FIXVERIFY 15</v>
@@ -681,7 +681,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-06-06</v>
+        <v>2026-06-07</v>
       </c>
       <c r="B9" t="str">
         <v>FIXVERIFY 15</v>
@@ -716,7 +716,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-06-06</v>
+        <v>2026-06-07</v>
       </c>
       <c r="B10" t="str">
         <v>FIXVERIFY 15</v>
@@ -751,7 +751,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-06-06</v>
+        <v>2026-06-07</v>
       </c>
       <c r="B11" t="str">
         <v>FIXVERIFY 15</v>

</xml_diff>